<commit_message>
Add 2026-05-22 and 2026-05-25 旭志農場 data to 歩留り表
【Row 35】2026-05-22 伝票番号00792（50頭）
- 積載/風袋: 25500/19490 kg（正味 6010 kg）
- 平均枝重: 82.6 kg / 歩留: 68.8%
- 格付け: 極1・上41・中2・並6
- 上物率: 84%、単価: 625円

【Row 36】2026-05-25 伝票番号00859（100頭）
- 積載/風袋: 25440/13300 kg（正味 12140 kg）
- 平均枝重: 81.9 kg / 歩留: 67.5%
- 格付け: 極2・上83・中4・並10・外1
- 上物率: 85%、単価: 625円

https://claude.ai/code/session_014wje5eaFCU8zUmm3Upt5mp
</commit_message>
<xml_diff>
--- a/R8.旭志歩留り表.xlsx
+++ b/R8.旭志歩留り表.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9216" yWindow="0" windowWidth="13704" windowHeight="12108" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2952" yWindow="180" windowWidth="20280" windowHeight="12108" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="日々入力" sheetId="1" state="visible" r:id="rId1"/>
@@ -4482,9 +4482,22 @@
       <c r="R30" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="T30" s="48" t="n"/>
-      <c r="U30" s="48" t="n"/>
-      <c r="V30" s="48" t="n"/>
+      <c r="S30" s="0">
+        <f>SUM(N30:O30)</f>
+        <v/>
+      </c>
+      <c r="T30" s="48">
+        <f>IF(S30=0,"",(S30/E30*100))</f>
+        <v/>
+      </c>
+      <c r="U30" s="48">
+        <f>P30/E30*100</f>
+        <v/>
+      </c>
+      <c r="V30" s="48">
+        <f>Q30/E30*100</f>
+        <v/>
+      </c>
       <c r="X30" s="0" t="n">
         <v>681</v>
       </c>
@@ -4748,9 +4761,22 @@
       <c r="R32" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="T32" s="48" t="n"/>
-      <c r="U32" s="48" t="n"/>
-      <c r="V32" s="48" t="n"/>
+      <c r="S32" s="0">
+        <f>SUM(N32:O32)</f>
+        <v/>
+      </c>
+      <c r="T32" s="48">
+        <f>IF(S32=0,"",(S32/E32*100))</f>
+        <v/>
+      </c>
+      <c r="U32" s="48">
+        <f>P32/E32*100</f>
+        <v/>
+      </c>
+      <c r="V32" s="48">
+        <f>Q32/E32*100</f>
+        <v/>
+      </c>
       <c r="X32" s="0" t="n">
         <v>702</v>
       </c>
@@ -4893,9 +4919,22 @@
       <c r="R33" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="T33" s="48" t="n"/>
-      <c r="U33" s="48" t="n"/>
-      <c r="V33" s="48" t="n"/>
+      <c r="S33" s="0">
+        <f>SUM(N33:O33)</f>
+        <v/>
+      </c>
+      <c r="T33" s="48">
+        <f>IF(S33=0,"",(S33/E33*100))</f>
+        <v/>
+      </c>
+      <c r="U33" s="48">
+        <f>P33/E33*100</f>
+        <v/>
+      </c>
+      <c r="V33" s="48">
+        <f>Q33/E33*100</f>
+        <v/>
+      </c>
       <c r="X33" s="0" t="n">
         <v>719</v>
       </c>
@@ -5044,15 +5083,31 @@
       <c r="R34" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="S34" s="8" t="n"/>
-      <c r="T34" s="57" t="n"/>
-      <c r="U34" s="57" t="n"/>
-      <c r="V34" s="57" t="n"/>
-      <c r="W34" s="8" t="n"/>
+      <c r="S34" s="0">
+        <f>SUM(N34:O34)</f>
+        <v/>
+      </c>
+      <c r="T34" s="48">
+        <f>IF(S34=0,"",(S34/E34*100))</f>
+        <v/>
+      </c>
+      <c r="U34" s="48">
+        <f>P34/E34*100</f>
+        <v/>
+      </c>
+      <c r="V34" s="48">
+        <f>Q34/E34*100</f>
+        <v/>
+      </c>
       <c r="X34" s="8" t="n">
         <v>756</v>
       </c>
-      <c r="Y34" s="8" t="n"/>
+      <c r="Y34" s="8" t="n">
+        <v>769.73</v>
+      </c>
+      <c r="Z34" s="0" t="n">
+        <v>191.32</v>
+      </c>
       <c r="AA34" s="48" t="n"/>
       <c r="AB34" s="30" t="n">
         <v>2</v>
@@ -5148,24 +5203,24 @@
     </row>
     <row r="35" ht="18.6" customHeight="1" s="47" thickBot="1">
       <c r="C35" s="1" t="n">
-        <v>46155</v>
+        <v>46164</v>
       </c>
       <c r="D35" s="1">
         <f>TEXT(C35,"aaa")</f>
         <v/>
       </c>
       <c r="E35" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F35" s="0">
         <f>IF(E35=0,"",(E35-G35))</f>
         <v/>
       </c>
       <c r="H35" t="n">
-        <v>25970</v>
+        <v>25500</v>
       </c>
       <c r="I35" t="n">
-        <v>13770</v>
+        <v>19490</v>
       </c>
       <c r="J35" s="0">
         <f>IF(H35=0,"",(H35-I35))</f>
@@ -5176,28 +5231,28 @@
         <v/>
       </c>
       <c r="L35" t="n">
-        <v>81.8</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="M35" t="n">
-        <v>67.09999999999999</v>
+        <v>68.8</v>
+      </c>
+      <c r="N35" t="n">
+        <v>1</v>
       </c>
       <c r="O35" t="n">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="P35" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q35" t="n">
         <v>6</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>9</v>
-      </c>
-      <c r="R35" t="n">
-        <v>1</v>
       </c>
       <c r="S35">
         <f>SUM(N35:O35)</f>
         <v/>
       </c>
-      <c r="T35">
+      <c r="T35" s="48">
         <f>IF(S35=0,"",(S35/E35*100))</f>
         <v/>
       </c>
@@ -5214,7 +5269,7 @@
         <v/>
       </c>
       <c r="X35" t="n">
-        <v>771</v>
+        <v>625</v>
       </c>
       <c r="AA35" s="48" t="n"/>
       <c r="AB35" s="15" t="n">
@@ -5311,16 +5366,25 @@
     </row>
     <row r="36">
       <c r="C36" s="1" t="n">
-        <v>45779</v>
+        <v>46167</v>
       </c>
       <c r="D36" s="1">
         <f>TEXT(C36,"aaa")</f>
         <v/>
       </c>
+      <c r="E36" t="n">
+        <v>100</v>
+      </c>
       <c r="F36" s="0">
         <f>IF(E36=0,"",(E36-G36))</f>
         <v/>
       </c>
+      <c r="H36" t="n">
+        <v>25440</v>
+      </c>
+      <c r="I36" t="n">
+        <v>13300</v>
+      </c>
       <c r="J36" s="0">
         <f>IF(H36=0,"",(H36-I36))</f>
         <v/>
@@ -5329,9 +5393,50 @@
         <f>IF(E36=0,"",(J36/E36))</f>
         <v/>
       </c>
-      <c r="T36" s="48" t="n"/>
-      <c r="U36" s="48" t="n"/>
-      <c r="V36" s="48" t="n"/>
+      <c r="L36" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="M36" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="N36" t="n">
+        <v>2</v>
+      </c>
+      <c r="O36" t="n">
+        <v>83</v>
+      </c>
+      <c r="P36" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>10</v>
+      </c>
+      <c r="R36" t="n">
+        <v>1</v>
+      </c>
+      <c r="S36">
+        <f>SUM(N36:O36)</f>
+        <v/>
+      </c>
+      <c r="T36" s="48">
+        <f>IF(S36=0,"",(S36/E36*100))</f>
+        <v/>
+      </c>
+      <c r="U36" s="48">
+        <f>P36/E36*100</f>
+        <v/>
+      </c>
+      <c r="V36" s="48">
+        <f>Q36/E36*100</f>
+        <v/>
+      </c>
+      <c r="W36">
+        <f>R36/E36*100</f>
+        <v/>
+      </c>
+      <c r="X36" t="n">
+        <v>625</v>
+      </c>
       <c r="AB36" s="30" t="inlineStr">
         <is>
           <t>total</t>
@@ -5446,6 +5551,7 @@
         <f>IF(E37=0,"",(J37/E37))</f>
         <v/>
       </c>
+      <c r="T37" s="48" t="n"/>
       <c r="U37" s="48" t="n"/>
       <c r="V37" s="48" t="n"/>
       <c r="AB37" s="12" t="inlineStr">
@@ -5485,6 +5591,7 @@
         <v/>
       </c>
       <c r="R38" s="48" t="n"/>
+      <c r="T38" s="48" t="n"/>
       <c r="U38" s="48" t="n"/>
       <c r="V38" s="48" t="n"/>
       <c r="AB38" s="31" t="inlineStr">
@@ -5565,10 +5672,30 @@
       <c r="R39" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="U39" s="48" t="n"/>
-      <c r="V39" s="48" t="n"/>
+      <c r="S39" s="0">
+        <f>SUM(N39:O39)</f>
+        <v/>
+      </c>
+      <c r="T39" s="48">
+        <f>IF(S39=0,"",(S39/E39*100))</f>
+        <v/>
+      </c>
+      <c r="U39" s="48">
+        <f>P39/E39*100</f>
+        <v/>
+      </c>
+      <c r="V39" s="48">
+        <f>Q39/E39*100</f>
+        <v/>
+      </c>
       <c r="X39" s="0" t="n">
         <v>734</v>
+      </c>
+      <c r="Y39" s="0" t="n">
+        <v>859.05</v>
+      </c>
+      <c r="Z39" s="0" t="n">
+        <v>185.3</v>
       </c>
     </row>
     <row r="40">
@@ -5618,10 +5745,30 @@
       <c r="R40" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="U40" s="48" t="n"/>
-      <c r="V40" s="48" t="n"/>
+      <c r="S40" s="0">
+        <f>SUM(N40:O40)</f>
+        <v/>
+      </c>
+      <c r="T40" s="48">
+        <f>IF(S40=0,"",(S40/E40*100))</f>
+        <v/>
+      </c>
+      <c r="U40" s="48">
+        <f>P40/E40*100</f>
+        <v/>
+      </c>
+      <c r="V40" s="48">
+        <f>Q40/E40*100</f>
+        <v/>
+      </c>
       <c r="X40" s="0" t="n">
         <v>737</v>
+      </c>
+      <c r="Y40" s="0" t="n">
+        <v>838.6799999999999</v>
+      </c>
+      <c r="Z40" s="0" t="n">
+        <v>186.3</v>
       </c>
     </row>
     <row r="41">
@@ -5677,10 +5824,30 @@
       <c r="R41" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="U41" s="48" t="n"/>
-      <c r="V41" s="48" t="n"/>
+      <c r="S41" s="0">
+        <f>SUM(N41:O41)</f>
+        <v/>
+      </c>
+      <c r="T41" s="48">
+        <f>IF(S41=0,"",(S41/E41*100))</f>
+        <v/>
+      </c>
+      <c r="U41" s="48">
+        <f>P41/E41*100</f>
+        <v/>
+      </c>
+      <c r="V41" s="48">
+        <f>Q41/E41*100</f>
+        <v/>
+      </c>
       <c r="X41" s="0" t="n">
         <v>759</v>
+      </c>
+      <c r="Y41" s="0" t="n">
+        <v>851.3099999999999</v>
+      </c>
+      <c r="Z41" s="0" t="n">
+        <v>181.43</v>
       </c>
     </row>
     <row r="42">
@@ -5703,6 +5870,7 @@
         <f>IF(E42=0,"",(J42/E42))</f>
         <v/>
       </c>
+      <c r="T42" s="48" t="n"/>
       <c r="U42" s="48" t="n"/>
       <c r="V42" s="48" t="n"/>
     </row>
@@ -5750,8 +5918,22 @@
       <c r="R43" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="U43" s="48" t="n"/>
-      <c r="V43" s="48" t="n"/>
+      <c r="S43" s="0">
+        <f>SUM(N43:O43)</f>
+        <v/>
+      </c>
+      <c r="T43" s="48">
+        <f>IF(S43=0,"",(S43/E43*100))</f>
+        <v/>
+      </c>
+      <c r="U43" s="48">
+        <f>P43/E43*100</f>
+        <v/>
+      </c>
+      <c r="V43" s="48">
+        <f>Q43/E43*100</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="C44" s="1" t="n">
@@ -5773,6 +5955,7 @@
         <f>IF(E44=0,"",(J44/E44))</f>
         <v/>
       </c>
+      <c r="T44" s="48" t="n"/>
       <c r="U44" s="48" t="n"/>
       <c r="V44" s="48" t="n"/>
     </row>
@@ -5823,10 +6006,30 @@
       <c r="R45" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="U45" s="48" t="n"/>
-      <c r="V45" s="48" t="n"/>
+      <c r="S45" s="0">
+        <f>SUM(N45:O45)</f>
+        <v/>
+      </c>
+      <c r="T45" s="48">
+        <f>IF(S45=0,"",(S45/E45*100))</f>
+        <v/>
+      </c>
+      <c r="U45" s="48">
+        <f>P45/E45*100</f>
+        <v/>
+      </c>
+      <c r="V45" s="48">
+        <f>Q45/E45*100</f>
+        <v/>
+      </c>
       <c r="X45" s="0" t="n">
         <v>754</v>
+      </c>
+      <c r="Y45" s="0" t="n">
+        <v>874.84</v>
+      </c>
+      <c r="Z45" s="0" t="n">
+        <v>180.58</v>
       </c>
     </row>
     <row r="46">
@@ -5876,10 +6079,30 @@
       <c r="R46" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="U46" s="48" t="n"/>
-      <c r="V46" s="48" t="n"/>
+      <c r="S46" s="0">
+        <f>SUM(N46:O46)</f>
+        <v/>
+      </c>
+      <c r="T46" s="48">
+        <f>IF(S46=0,"",(S46/E46*100))</f>
+        <v/>
+      </c>
+      <c r="U46" s="48">
+        <f>P46/E46*100</f>
+        <v/>
+      </c>
+      <c r="V46" s="48">
+        <f>Q46/E46*100</f>
+        <v/>
+      </c>
       <c r="X46" s="0" t="n">
         <v>771</v>
+      </c>
+      <c r="Y46" s="0" t="n">
+        <v>1013.78</v>
+      </c>
+      <c r="Z46" s="0" t="n">
+        <v>166.96</v>
       </c>
     </row>
     <row r="47">
@@ -5929,10 +6152,30 @@
       <c r="R47" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="U47" s="48" t="n"/>
-      <c r="V47" s="48" t="n"/>
+      <c r="S47" s="0">
+        <f>SUM(N47:O47)</f>
+        <v/>
+      </c>
+      <c r="T47" s="48">
+        <f>IF(S47=0,"",(S47/E47*100))</f>
+        <v/>
+      </c>
+      <c r="U47" s="48">
+        <f>P47/E47*100</f>
+        <v/>
+      </c>
+      <c r="V47" s="48">
+        <f>Q47/E47*100</f>
+        <v/>
+      </c>
       <c r="X47" s="0" t="n">
         <v>749</v>
+      </c>
+      <c r="Y47" s="0" t="n">
+        <v>821.72</v>
+      </c>
+      <c r="Z47" s="0" t="n">
+        <v>182.46</v>
       </c>
     </row>
     <row r="48">
@@ -5955,6 +6198,7 @@
         <f>IF(E48=0,"",(J48/E48))</f>
         <v/>
       </c>
+      <c r="T48" s="48" t="n"/>
       <c r="U48" s="48" t="n"/>
       <c r="V48" s="48" t="n"/>
     </row>
@@ -5966,10 +6210,19 @@
         <f>TEXT(C49,"aaa")</f>
         <v/>
       </c>
+      <c r="E49" s="0" t="n">
+        <v>100</v>
+      </c>
       <c r="F49" s="0">
         <f>IF(E49=0,"",(E49-G49))</f>
         <v/>
       </c>
+      <c r="H49" s="0" t="n">
+        <v>26330</v>
+      </c>
+      <c r="I49" s="0" t="n">
+        <v>13450</v>
+      </c>
       <c r="J49" s="0">
         <f>IF(H49=0,"",(H49-I49))</f>
         <v/>
@@ -5978,8 +6231,49 @@
         <f>IF(E49=0,"",(J49/E49))</f>
         <v/>
       </c>
-      <c r="U49" s="48" t="n"/>
-      <c r="V49" s="48" t="n"/>
+      <c r="L49" s="0" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="M49" s="0" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="O49" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="P49" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q49" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="R49" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="S49" s="0">
+        <f>SUM(N49:O49)</f>
+        <v/>
+      </c>
+      <c r="T49" s="48">
+        <f>IF(S49=0,"",(S49/E49*100))</f>
+        <v/>
+      </c>
+      <c r="U49" s="48">
+        <f>P49/E49*100</f>
+        <v/>
+      </c>
+      <c r="V49" s="48">
+        <f>Q49/E49*100</f>
+        <v/>
+      </c>
+      <c r="X49" s="0" t="n">
+        <v>653</v>
+      </c>
+      <c r="Y49" s="0" t="n">
+        <v>962.34</v>
+      </c>
+      <c r="Z49" s="0" t="n">
+        <v>174.38</v>
+      </c>
     </row>
     <row r="50">
       <c r="C50" s="1" t="n">
@@ -6001,6 +6295,7 @@
         <f>IF(E50=0,"",(J50/E50))</f>
         <v/>
       </c>
+      <c r="T50" s="48" t="n"/>
       <c r="U50" s="48" t="n"/>
       <c r="V50" s="48" t="n"/>
     </row>
@@ -6024,6 +6319,7 @@
         <f>IF(E51=0,"",(J51/E51))</f>
         <v/>
       </c>
+      <c r="T51" s="48" t="n"/>
       <c r="U51" s="48" t="n"/>
       <c r="V51" s="48" t="n"/>
     </row>
@@ -6035,10 +6331,19 @@
         <f>TEXT(C52,"aaa")</f>
         <v/>
       </c>
+      <c r="E52" s="0" t="n">
+        <v>100</v>
+      </c>
       <c r="F52" s="0">
         <f>IF(E52=0,"",(E52-G52))</f>
         <v/>
       </c>
+      <c r="H52" s="0" t="n">
+        <v>26020</v>
+      </c>
+      <c r="I52" s="0" t="n">
+        <v>13840</v>
+      </c>
       <c r="J52" s="0">
         <f>IF(H52=0,"",(H52-I52))</f>
         <v/>
@@ -6047,8 +6352,46 @@
         <f>IF(E52=0,"",(J52/E52))</f>
         <v/>
       </c>
-      <c r="U52" s="48" t="n"/>
-      <c r="V52" s="48" t="n"/>
+      <c r="L52" s="0" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="N52" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="O52" s="0" t="n">
+        <v>73</v>
+      </c>
+      <c r="P52" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q52" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="S52" s="0">
+        <f>SUM(N52:O52)</f>
+        <v/>
+      </c>
+      <c r="T52" s="48">
+        <f>IF(S52=0,"",(S52/E52*100))</f>
+        <v/>
+      </c>
+      <c r="U52" s="48">
+        <f>P52/E52*100</f>
+        <v/>
+      </c>
+      <c r="V52" s="48">
+        <f>Q52/E52*100</f>
+        <v/>
+      </c>
+      <c r="X52" s="0" t="n">
+        <v>693</v>
+      </c>
+      <c r="Y52" s="0" t="n">
+        <v>951.34</v>
+      </c>
+      <c r="Z52" s="0" t="n">
+        <v>176.82</v>
+      </c>
     </row>
     <row r="53">
       <c r="C53" s="1" t="n">
@@ -6058,10 +6401,22 @@
         <f>TEXT(C53,"aaa")</f>
         <v/>
       </c>
+      <c r="E53" s="0" t="n">
+        <v>100</v>
+      </c>
       <c r="F53" s="0">
         <f>IF(E53=0,"",(E53-G53))</f>
         <v/>
       </c>
+      <c r="G53" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" s="0" t="n">
+        <v>26120</v>
+      </c>
+      <c r="I53" s="0" t="n">
+        <v>13750</v>
+      </c>
       <c r="J53" s="0">
         <f>IF(H53=0,"",(H53-I53))</f>
         <v/>
@@ -6070,8 +6425,52 @@
         <f>IF(E53=0,"",(J53/E53))</f>
         <v/>
       </c>
-      <c r="U53" s="48" t="n"/>
-      <c r="V53" s="48" t="n"/>
+      <c r="L53" s="0" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="M53" s="0" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="N53" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="O53" s="0" t="n">
+        <v>66</v>
+      </c>
+      <c r="P53" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q53" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="R53" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S53" s="0">
+        <f>SUM(N53:O53)</f>
+        <v/>
+      </c>
+      <c r="T53" s="48">
+        <f>IF(S53=0,"",(S53/E53*100))</f>
+        <v/>
+      </c>
+      <c r="U53" s="48">
+        <f>P53/E53*100</f>
+        <v/>
+      </c>
+      <c r="V53" s="48">
+        <f>Q53/E53*100</f>
+        <v/>
+      </c>
+      <c r="X53" s="0" t="n">
+        <v>686</v>
+      </c>
+      <c r="Y53" s="0" t="n">
+        <v>810.58</v>
+      </c>
+      <c r="Z53" s="0" t="n">
+        <v>184.4</v>
+      </c>
     </row>
     <row r="54">
       <c r="C54" s="1" t="n">
@@ -6081,10 +6480,19 @@
         <f>TEXT(C54,"aaa")</f>
         <v/>
       </c>
+      <c r="E54" s="0" t="n">
+        <v>100</v>
+      </c>
       <c r="F54" s="0">
         <f>IF(E54=0,"",(E54-G54))</f>
         <v/>
       </c>
+      <c r="H54" s="0" t="n">
+        <v>25650</v>
+      </c>
+      <c r="I54" s="0" t="n">
+        <v>13320</v>
+      </c>
       <c r="J54" s="0">
         <f>IF(H54=0,"",(H54-I54))</f>
         <v/>
@@ -6093,21 +6501,62 @@
         <f>IF(E54=0,"",(J54/E54))</f>
         <v/>
       </c>
-      <c r="U54" s="48" t="n"/>
-      <c r="V54" s="48" t="n"/>
+      <c r="L54" s="0" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="M54" s="0" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="O54" s="0" t="n">
+        <v>74</v>
+      </c>
+      <c r="P54" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q54" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="S54" s="0">
+        <f>SUM(N54:O54)</f>
+        <v/>
+      </c>
+      <c r="T54" s="48">
+        <f>IF(S54=0,"",(S54/E54*100))</f>
+        <v/>
+      </c>
+      <c r="U54" s="48">
+        <f>P54/E54*100</f>
+        <v/>
+      </c>
+      <c r="V54" s="48">
+        <f>Q54/E54*100</f>
+        <v/>
+      </c>
+      <c r="X54" s="0" t="n">
+        <v>690</v>
+      </c>
     </row>
     <row r="55">
       <c r="C55" s="1" t="n">
-        <v>45798</v>
+        <v>45797</v>
       </c>
       <c r="D55" s="1">
         <f>TEXT(C55,"aaa")</f>
         <v/>
       </c>
+      <c r="E55" s="0" t="n">
+        <v>100</v>
+      </c>
       <c r="F55" s="0">
         <f>IF(E55=0,"",(E55-G55))</f>
         <v/>
       </c>
+      <c r="H55" s="0" t="n">
+        <v>25700</v>
+      </c>
+      <c r="I55" s="0" t="n">
+        <v>13190</v>
+      </c>
       <c r="J55" s="0">
         <f>IF(H55=0,"",(H55-I55))</f>
         <v/>
@@ -6116,8 +6565,43 @@
         <f>IF(E55=0,"",(J55/E55))</f>
         <v/>
       </c>
-      <c r="U55" s="48" t="n"/>
-      <c r="V55" s="48" t="n"/>
+      <c r="L55" s="0" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="M55" s="0" t="n">
+        <v>68</v>
+      </c>
+      <c r="O55" s="0" t="n">
+        <v>74</v>
+      </c>
+      <c r="P55" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q55" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="R55" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="S55" s="0">
+        <f>SUM(N55:O55)</f>
+        <v/>
+      </c>
+      <c r="T55" s="48">
+        <f>IF(S55=0,"",(S55/E55*100))</f>
+        <v/>
+      </c>
+      <c r="U55" s="48">
+        <f>P55/E55*100</f>
+        <v/>
+      </c>
+      <c r="V55" s="48">
+        <f>Q55/E55*100</f>
+        <v/>
+      </c>
+      <c r="X55" s="0" t="n">
+        <v>659</v>
+      </c>
     </row>
     <row r="56">
       <c r="C56" s="1" t="n">
@@ -6139,6 +6623,7 @@
         <f>IF(E56=0,"",(J56/E56))</f>
         <v/>
       </c>
+      <c r="T56" s="48" t="n"/>
       <c r="U56" s="48" t="n"/>
       <c r="V56" s="48" t="n"/>
     </row>
@@ -6162,6 +6647,7 @@
         <f>IF(E57=0,"",(J57/E57))</f>
         <v/>
       </c>
+      <c r="T57" s="48" t="n"/>
       <c r="U57" s="48" t="n"/>
       <c r="V57" s="48" t="n"/>
     </row>
@@ -6185,6 +6671,7 @@
         <f>IF(E58=0,"",(J58/E58))</f>
         <v/>
       </c>
+      <c r="T58" s="48" t="n"/>
       <c r="U58" s="48" t="n"/>
       <c r="V58" s="48" t="n"/>
     </row>
@@ -6208,6 +6695,7 @@
         <f>IF(E59=0,"",(J59/E59))</f>
         <v/>
       </c>
+      <c r="T59" s="48" t="n"/>
       <c r="U59" s="48" t="n"/>
       <c r="V59" s="48" t="n"/>
     </row>
@@ -6231,6 +6719,7 @@
         <f>IF(E60=0,"",(J60/E60))</f>
         <v/>
       </c>
+      <c r="T60" s="48" t="n"/>
       <c r="U60" s="48" t="n"/>
       <c r="V60" s="48" t="n"/>
     </row>
@@ -6254,6 +6743,7 @@
         <f>IF(E61=0,"",(J61/E61))</f>
         <v/>
       </c>
+      <c r="T61" s="48" t="n"/>
       <c r="U61" s="48" t="n"/>
       <c r="V61" s="48" t="n"/>
     </row>
@@ -6277,6 +6767,7 @@
         <f>IF(E62=0,"",(J62/E62))</f>
         <v/>
       </c>
+      <c r="T62" s="48" t="n"/>
       <c r="U62" s="48" t="n"/>
       <c r="V62" s="48" t="n"/>
     </row>
@@ -6300,6 +6791,7 @@
         <f>IF(E63=0,"",(J63/E63))</f>
         <v/>
       </c>
+      <c r="T63" s="48" t="n"/>
       <c r="U63" s="48" t="n"/>
       <c r="V63" s="48" t="n"/>
     </row>
@@ -6323,6 +6815,7 @@
         <f>IF(E64=0,"",(J64/E64))</f>
         <v/>
       </c>
+      <c r="T64" s="48" t="n"/>
       <c r="U64" s="48" t="n"/>
       <c r="V64" s="48" t="n"/>
     </row>
@@ -6359,6 +6852,9 @@
       <c r="P65" s="8" t="n"/>
       <c r="Q65" s="8" t="n"/>
       <c r="R65" s="8" t="n"/>
+      <c r="T65" s="48" t="n"/>
+      <c r="U65" s="48" t="n"/>
+      <c r="V65" s="48" t="n"/>
       <c r="X65" s="8" t="n"/>
       <c r="Y65" s="8" t="n"/>
     </row>

</xml_diff>

<commit_message>
Restore 2026-05-13 entry and reorder May shipments chronologically
The 2026-05-13 shipment (100頭, 伝票00343) was lost when the file was
replaced with a fresh template copy in a later update. Re-enter it at
row 35 and shift 2026-05-22 / 2026-05-25 to rows 36-37 so all three
May entries are in date order. Grading-count sums verified against
head counts (100/50/100).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014wje5eaFCU8zUmm3Upt5mp
</commit_message>
<xml_diff>
--- a/R8.旭志歩留り表.xlsx
+++ b/R8.旭志歩留り表.xlsx
@@ -5203,24 +5203,24 @@
     </row>
     <row r="35" ht="18.6" customHeight="1" s="47" thickBot="1">
       <c r="C35" s="1" t="n">
-        <v>46164</v>
+        <v>46155</v>
       </c>
       <c r="D35" s="1">
         <f>TEXT(C35,"aaa")</f>
         <v/>
       </c>
-      <c r="E35" t="n">
-        <v>50</v>
+      <c r="E35" s="0" t="n">
+        <v>100</v>
       </c>
       <c r="F35" s="0">
         <f>IF(E35=0,"",(E35-G35))</f>
         <v/>
       </c>
-      <c r="H35" t="n">
-        <v>25500</v>
-      </c>
-      <c r="I35" t="n">
-        <v>19490</v>
+      <c r="H35" s="0" t="n">
+        <v>25970</v>
+      </c>
+      <c r="I35" s="0" t="n">
+        <v>13770</v>
       </c>
       <c r="J35" s="0">
         <f>IF(H35=0,"",(H35-I35))</f>
@@ -5230,25 +5230,26 @@
         <f>IF(E35=0,"",(J35/E35))</f>
         <v/>
       </c>
-      <c r="L35" t="n">
-        <v>82.59999999999999</v>
-      </c>
-      <c r="M35" t="n">
-        <v>68.8</v>
-      </c>
-      <c r="N35" t="n">
+      <c r="L35" s="0" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="M35" s="0" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="N35" s="0" t="n"/>
+      <c r="O35" s="0" t="n">
+        <v>84</v>
+      </c>
+      <c r="P35" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q35" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="R35" t="n">
         <v>1</v>
       </c>
-      <c r="O35" t="n">
-        <v>41</v>
-      </c>
-      <c r="P35" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>6</v>
-      </c>
-      <c r="S35">
+      <c r="S35" s="0">
         <f>SUM(N35:O35)</f>
         <v/>
       </c>
@@ -5264,12 +5265,12 @@
         <f>Q35/E35*100</f>
         <v/>
       </c>
-      <c r="W35">
+      <c r="W35" s="0">
         <f>R35/E35*100</f>
         <v/>
       </c>
-      <c r="X35" t="n">
-        <v>625</v>
+      <c r="X35" s="0" t="n">
+        <v>771</v>
       </c>
       <c r="AA35" s="48" t="n"/>
       <c r="AB35" s="15" t="n">
@@ -5366,24 +5367,24 @@
     </row>
     <row r="36">
       <c r="C36" s="1" t="n">
-        <v>46167</v>
+        <v>46164</v>
       </c>
       <c r="D36" s="1">
         <f>TEXT(C36,"aaa")</f>
         <v/>
       </c>
-      <c r="E36" t="n">
-        <v>100</v>
+      <c r="E36" s="0" t="n">
+        <v>50</v>
       </c>
       <c r="F36" s="0">
         <f>IF(E36=0,"",(E36-G36))</f>
         <v/>
       </c>
-      <c r="H36" t="n">
-        <v>25440</v>
-      </c>
-      <c r="I36" t="n">
-        <v>13300</v>
+      <c r="H36" s="0" t="n">
+        <v>25500</v>
+      </c>
+      <c r="I36" s="0" t="n">
+        <v>19490</v>
       </c>
       <c r="J36" s="0">
         <f>IF(H36=0,"",(H36-I36))</f>
@@ -5393,28 +5394,26 @@
         <f>IF(E36=0,"",(J36/E36))</f>
         <v/>
       </c>
-      <c r="L36" t="n">
-        <v>81.90000000000001</v>
-      </c>
-      <c r="M36" t="n">
-        <v>67.5</v>
-      </c>
-      <c r="N36" t="n">
+      <c r="L36" s="0" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="M36" s="0" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="N36" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="O36" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="P36" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="O36" t="n">
-        <v>83</v>
-      </c>
-      <c r="P36" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>10</v>
-      </c>
-      <c r="R36" t="n">
-        <v>1</v>
-      </c>
-      <c r="S36">
+      <c r="Q36" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="R36" s="0" t="n"/>
+      <c r="S36" s="0">
         <f>SUM(N36:O36)</f>
         <v/>
       </c>
@@ -5430,11 +5429,11 @@
         <f>Q36/E36*100</f>
         <v/>
       </c>
-      <c r="W36">
+      <c r="W36" s="0">
         <f>R36/E36*100</f>
         <v/>
       </c>
-      <c r="X36" t="n">
+      <c r="X36" s="0" t="n">
         <v>625</v>
       </c>
       <c r="AB36" s="30" t="inlineStr">
@@ -5533,16 +5532,25 @@
     </row>
     <row r="37">
       <c r="C37" s="1" t="n">
-        <v>45780</v>
+        <v>46167</v>
       </c>
       <c r="D37" s="1">
         <f>TEXT(C37,"aaa")</f>
         <v/>
       </c>
+      <c r="E37" t="n">
+        <v>100</v>
+      </c>
       <c r="F37" s="0">
         <f>IF(E37=0,"",(E37-G37))</f>
         <v/>
       </c>
+      <c r="H37" t="n">
+        <v>25440</v>
+      </c>
+      <c r="I37" t="n">
+        <v>13300</v>
+      </c>
       <c r="J37" s="0">
         <f>IF(H37=0,"",(H37-I37))</f>
         <v/>
@@ -5551,9 +5559,50 @@
         <f>IF(E37=0,"",(J37/E37))</f>
         <v/>
       </c>
-      <c r="T37" s="48" t="n"/>
-      <c r="U37" s="48" t="n"/>
-      <c r="V37" s="48" t="n"/>
+      <c r="L37" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="M37" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="N37" t="n">
+        <v>2</v>
+      </c>
+      <c r="O37" t="n">
+        <v>83</v>
+      </c>
+      <c r="P37" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>10</v>
+      </c>
+      <c r="R37" t="n">
+        <v>1</v>
+      </c>
+      <c r="S37">
+        <f>SUM(N37:O37)</f>
+        <v/>
+      </c>
+      <c r="T37" s="48">
+        <f>IF(S37=0,"",(S37/E37*100))</f>
+        <v/>
+      </c>
+      <c r="U37" s="48">
+        <f>P37/E37*100</f>
+        <v/>
+      </c>
+      <c r="V37" s="48">
+        <f>Q37/E37*100</f>
+        <v/>
+      </c>
+      <c r="W37">
+        <f>R37/E37*100</f>
+        <v/>
+      </c>
+      <c r="X37" t="n">
+        <v>625</v>
+      </c>
       <c r="AB37" s="12" t="inlineStr">
         <is>
           <t>R7</t>

</xml_diff>